<commit_message>
T-0033 (1/2) — Souche gabarit-pilotage-mission.xlsx régénérée propre (canon)
Remplacement du binaire souche canon par la sortie du générateur (promotion d'un binaire
socle : le corps est remplacé, l'historique Git porte la trace). Aucun autre contrat touché.

Retire la pollution S35 (lignes MIS-EXEMPLE / jane.doe@allia-consulting.com / F-EXEMPLE-001,
statuts non accentués « a valider »/« a emettre »). Les 3 tables sont désormais en-têtes seuls
(ref A1:D1 / A1:E1 / A1:G1), statuts de référence accentués en listes de validation.
Auto-vérification (a)..(e) verte — sortie complète dans la description de la PR.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/contrats/socle/gabarit-pilotage-mission.xlsx
+++ b/contrats/socle/gabarit-pilotage-mission.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legende" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Affectations" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Imputations" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Echeancier" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Legende" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Affectations" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Imputations" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Echeancier" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,29 +33,11 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00808080"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00C00000"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -64,7 +46,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -74,11 +56,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -94,19 +71,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -183,119 +156,9 @@
 </styleSheet>
 </file>
 
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Gabarit</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>id stable de la mission</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>identifiant Entra (couture Ressources-Profil)</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>1er du mois — granularite mensuelle</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>budget de charge du mois</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Gabarit</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>id stable</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>identifiant Entra</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>1er du mois</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>saisie du collaborateur</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>'a valider' / 'valide' — ecrit par le responsable via le cockpit</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Gabarit</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>id stable de la facture</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>id stable</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>1er du mois de rattachement du CA</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>euros</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>date d'echeance</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>'a emettre' / 'emise' / 'payee'</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>URL du PDF dans le depot Teams de la mission</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_Affectations" displayName="T_Affectations" ref="A1:D2" headerRowCount="1">
-  <autoFilter ref="A1:D2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_Affectations" displayName="T_Affectations" ref="A1:D1" headerRowCount="1">
+  <autoFilter ref="A1:D1"/>
   <tableColumns count="4">
     <tableColumn id="1" name="CodeMission"/>
     <tableColumn id="2" name="Ressource"/>
@@ -307,8 +170,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T_Imputations" displayName="T_Imputations" ref="A1:E2" headerRowCount="1">
-  <autoFilter ref="A1:E2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T_Imputations" displayName="T_Imputations" ref="A1:E1" headerRowCount="1">
+  <autoFilter ref="A1:E1"/>
   <tableColumns count="5">
     <tableColumn id="1" name="CodeMission"/>
     <tableColumn id="2" name="Ressource"/>
@@ -321,8 +184,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T_Echeancier" displayName="T_Echeancier" ref="A1:G2" headerRowCount="1">
-  <autoFilter ref="A1:G2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T_Echeancier" displayName="T_Echeancier" ref="A1:G1" headerRowCount="1">
+  <autoFilter ref="A1:G1"/>
   <tableColumns count="7">
     <tableColumn id="1" name="NumFacture"/>
     <tableColumn id="2" name="CodeMission"/>
@@ -625,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -639,67 +502,75 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Instancier ce gabarit en pilotage-&lt;CodeMission&gt;.xlsx dans l'espace de la mission, a la bascule « Gagnee » de l'opportunite.</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Souche canon (modele-donnees.md §5.2). Instanciée par l'agent, une par mission, en gabarit-&lt;CodeMission&gt;.xlsx (instanciation SYSTÉMATIQUE et machine, §5.6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Trois onglets. Les noms de tables et les en-têtes de colonnes sont FIGÉS (§5.2) : ne jamais les renommer.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Trois onglets a remplir. Les en-tetes de colonnes et les noms de tables sont figes : ne pas les renommer.</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Les tables sont livrées VIDES (en-têtes seuls). Saisir les données réelles sous la ligne d'en-tête ; aucune ligne d'exemple à remplacer.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>La premiere ligne grisee de chaque table est un EXEMPLE : la remplacer par vos donnees reelles.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Aucun cout, taux ou salaire ne figure dans ce fichier (regle du modele : les couts restent au consolide central).</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Aucun coût, taux ni salaire ne figure dans ce fichier : les coûts vivent dans le référentiel de coûts à audience restreinte (§5.3), jamais dans les gabarits mission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>T_Affectations</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>T_Affectations</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>prevoir le staffing : qui, quel mois, combien de jours prevus.</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>prévoir le staffing : qui, quel mois, combien de jours prévus.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>T_Imputations</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>declarer le realise : jours realises par ressource et par mois + statut de validation.</t>
-        </is>
-      </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>déclarer le réalisé : jours réalisés par ressource et par mois + statut de validation (« à valider » / « validé »).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>T_Echeancier</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>plan de facturation : factures, mois de CA, montant HT, echeance, statut, lien PDF.</t>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>plan de facturation : facture, mois de CA, montant HT, échéance, statut (« à émettre » / « émise » / « payée »), lien PDF.</t>
         </is>
       </c>
     </row>
@@ -714,60 +585,39 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" style="3" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>CodeMission</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Ressource</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Mois</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>JoursPrevus</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>MIS-EXEMPLE</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>jane.doe@allia-consulting.com</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="n">
-        <v>12</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
@@ -780,71 +630,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" style="3" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>CodeMission</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Ressource</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Mois</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>JoursRealises</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>StatutValidation</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>MIS-EXEMPLE</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>jane.doe@allia-consulting.com</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>a valider</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"à valider,validé"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
@@ -857,89 +686,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" style="3" min="3" max="3"/>
+    <col width="15" customWidth="1" style="5" min="4" max="4"/>
+    <col width="14" customWidth="1" style="3" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>NumFacture</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>CodeMission</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>MoisCA</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>MontantHT</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Echeance</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Statut</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>LienFacture</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>F-EXEMPLE-001</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>MIS-EXEMPLE</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="D2" s="9" t="n">
-        <v>18000</v>
-      </c>
-      <c r="E2" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>a emettre</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr"/>
-    </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"à émettre,émise,payée"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>

</xml_diff>